<commit_message>
Añadir pestaña 6 · Metodología (CENIA v2) a la planilla final
Embebe la metodología final acordada con el CENIA dentro de la planilla
(antes solo estaba en archivos externos): tabla variable por variable con
su normalización y la columna de la pestaña 1 que la alimenta, el detalle
de los 3 sub-componentes de Organización Convocante (amplitud gubernamental
÷3 + amplitud no gubernamental ÷4 + co-convocatoria por máximo relativo) y
las notas clave (universidades públicas = Universidad, co-convocatoria
deduplicada, conteo de todas las elegibles). Guía y navegación actualizadas
de 5 a 6 pestañas.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/planilla_ILIA2026_SIMPLE.xlsx
+++ b/data/gates/planilla_ILIA2026_SIMPLE.xlsx
@@ -12,6 +12,7 @@
     <sheet name="3 · Excluidos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="4 · Evidencia y fuentes" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5 · Instrucciones" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="6 · Metodología (CENIA v2)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 · Casos (entran+dudosos)'!$A$1:$X$45</definedName>
@@ -26,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +45,15 @@
     <font>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="8">
@@ -84,7 +94,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -106,11 +116,44 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -152,6 +195,26 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -11284,7 +11347,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>Planilla con 5 pestañas. 44 casos entran/dudosos · 63 excluidos · 107 en total. Tras dedup e-Cidadania: 43 iniciativas.</t>
+          <t>Planilla con 6 pestañas. 44 casos entran/dudosos · 63 excluidos · 107 en total. Tras dedup e-Cidadania: 43 iniciativas.</t>
         </is>
       </c>
     </row>
@@ -11296,7 +11359,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Pestaña 1 = trabajo y cálculo · 2 = qué decidir a mano · 3 = excluidos (referencia) · 4 = evidencia/citas · 5 = esta guía.</t>
+          <t>Pestaña 1 = trabajo y cálculo · 2 = qué decidir a mano · 3 = excluidos (referencia) · 4 = evidencia/citas · 5 = esta guía · 6 = metodología CENIA v2.</t>
         </is>
       </c>
     </row>
@@ -11431,4 +11494,351 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>METODOLOGÍA FINAL — IA en Participación Ciudadana (CENIA v2 · jun-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Indicador = (Sub-Indicador de Uso + Sub-Indicador de Desarrollo) / 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr"/>
+      <c r="B3" s="13" t="inlineStr"/>
+      <c r="C3" s="13" t="inlineStr"/>
+      <c r="D3" s="13" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Sub-indicador</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Cómo se calcula (normalización)</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Columna en pestaña 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Uso de IA
+(promedio simple
+de 5 variables)</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Tipos de proceso</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>nº de tipos distintos ÷ 5 (máximo absoluto)</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Tipo de proceso</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="n"/>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Etapas de uso</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>nº de etapas distintas ÷ 4 (máximo absoluto)</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Etapas uso IA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="n"/>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Continuidad</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>nivel MÁXIMO verificado del país ÷ 3 · un 'anuncio' caduca a los 2 años sin implementación</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Nivel (0-3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="n"/>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Organización Convocante</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>promedio de 3 sub-componentes co-iguales (ver detalle abajo)</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Convocante (7-cat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="n"/>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Cantidad de iniciativas</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>nº de TODAS las iniciativas elegibles del país · umbrales fijos 0→0 · 1-3→25 · 4-6→50 · 7-9→75 · 10+→100</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>1 fila = 1 iniciativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Desarrollo de IA
+(idéntico a 2025)</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Desarrollador</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>nacional / internacional × 4 tipos de actor · máximo relativo</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Tipo desarrollador IA · Origen</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="n"/>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Tipos de IA</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>nº de sistemas de IA distintos · máximo relativo</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Tipos/familia IA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr"/>
+      <c r="B12" s="13" t="inlineStr"/>
+      <c r="C12" s="13" t="inlineStr"/>
+      <c r="D12" s="13" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>ORGANIZACIÓN CONVOCANTE — 3 sub-componentes co-iguales · valor de la variable = (1 + 2 + 3) / 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>1 · Amplitud gubernamental</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>nº de tipos gubernamentales distintos ÷ 3</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>gobierno local · gobierno nacional · otra institución pública</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>2 · Amplitud no gubernamental</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>nº de tipos no gubernamentales distintos ÷ 4</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>empresa · universidad · sociedad civil · organización internacional</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>3 · Co-convocatoria</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>nº de combinaciones distintas (conjuntos de ≥2 tipos que co-convocan una misma iniciativa) ÷ máximo relativo móvil del ciclo</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>combinaciones DEDUPLICADAS · una co-convocatoria de 4 actores = 1 combinación</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr"/>
+      <c r="B17" s="13" t="inlineStr"/>
+      <c r="C17" s="13" t="inlineStr"/>
+      <c r="D17" s="13" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>• Universidades públicas → cuentan como 'Universidad' (no gubernamental), NO como 'otra institución pública'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr"/>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>• Anotar TODOS los convocantes de cada iniciativa (no solo el principal): así se detecta la co-convocatoria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr"/>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>• El máximo relativo de co-convocatoria se recalcula en cada corrida del motor — no se fija a mano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr"/>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>• 'Cantidad' cuenta las iniciativas elegibles; los duplicados (Cuenta como iniciativa = NO) no se suman.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr"/>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>• El Sub-Indicador de Desarrollo es idéntico al de 2025 (no se modificó).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr"/>
+      <c r="B23" s="13" t="inlineStr"/>
+      <c r="C23" s="13" t="inlineStr"/>
+      <c r="D23" s="13" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>metodologia_final_CENIA_v2.xlsx · detalle de conformidad en conformidad_metodologia_CENIA.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="A5:A9"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="B20:D20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Embeber hallazgos de investigación en las DUDAs de revisión (TT/DO/CO DNP)
Investigación web dirigida sobre los 3 casos que el equipo dejó en DUDA:
- TT EngageTT: IA mixta — chatbot AskNDTS (explicador, no procesa aportes) activo;
  módulo Sensemaking de Go Vocal NO confirmado activado/anunciado para TT. DUDA real.
- CO DNP Diálogos: análisis de fondo manual/cualitativo; solo nubes de palabras +
  tabulación por sectores; sin NLP profundo ni ConTexto confirmado → recomiendo NO.
- DO CiudadanIA: solo atención/servicio; la 'participación' es co-diseñar la IA
  aportando datos, no consulta pública; sin módulo de participación → recomiendo NO.

Notas con hallazgo + recomendación + URL embebidas en la pestaña 2 (grupo C).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/planilla_ILIA2026_SIMPLE.xlsx
+++ b/data/gates/planilla_ILIA2026_SIMPLE.xlsx
@@ -5862,7 +5862,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>¿La IA de Go Vocal (Sensemaking) está ACTIVA o PLANEADA? Si está planeada, ENTRA.</t>
+          <t>IA MIXTA: chatbot AskNDTS (IA) activo que ayuda a ENTENDER el NDTS (facilitación/info, no procesa aportes). El módulo Sensemaking de Go Vocal existe pero NO se confirma activado ni anunciado para TT. Ministerio ahora MPAAI (Public Admin + AI). → DUDA: ¿basta el chatbot explicador como 'IA en el proceso'? Ver mdt.gov.tt (EngageTT + AskNDTS).</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -5901,7 +5901,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>¿Se usó NLP (p. ej. ConTexto del DNP) para sistematizar las 89.788 propuestas?</t>
+          <t>Análisis de fondo MANUAL/cualitativo (lectura + recurrencia, 7 categorías). Solo text-analytics ligero: nubes de palabras + tabulación por sectores (UCD). Sin NLP profundo ni ConTexto confirmado en los DRV → RECOMIENDO NO. Ver dialogosregionales.dnp.gov.co/resultados-dialogos.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>¿Tiene un módulo de participación (recoger aportes para decisiones), no solo atención/servicio?</t>
+          <t>Solo funciones de ATENCIÓN/SERVICIO; la 'participación' que menciona es co-diseñar la IA aportando datos, no consulta/decisión pública. No se halló módulo de participación → RECOMIENDO NO. Ver genia.ai/plataforma.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Regenerar planillas finales (interna + por país) con URLs verificadas
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/planilla_ILIA2026_SIMPLE.xlsx
+++ b/data/gates/planilla_ILIA2026_SIMPLE.xlsx
@@ -1996,7 +1996,7 @@
         <is>
           <t>https://www.bcn.cl/procesoconstituyente/cabildos2016/
 https://aclanthology.org/W17-5101/
-https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0267443</t>
+https://journals.plos.org/plosone/article?id=10.1371%2Fjournal.pone.0267443</t>
         </is>
       </c>
       <c r="X12" s="2" t="inlineStr">
@@ -2230,8 +2230,8 @@
       </c>
       <c r="W14" s="2" t="inlineStr">
         <is>
-          <t>https://participacion.digital.gob.cl/es-CL/folders/consultas-ciudadanas
-https://participacion.digital.gob.cl/projects/segunda-consulta-estrategia-de-gobierno-digital-2030</t>
+          <t>https://participacion.digital.gob.cl/projects/segunda-consulta-estrategia-de-gobierno-digital-2030
+https://participacion.digital.gob.cl/folders/consultas-ciudadanas</t>
         </is>
       </c>
       <c r="X14" s="2" t="inlineStr">
@@ -2345,8 +2345,8 @@
       </c>
       <c r="W15" s="2" t="inlineStr">
         <is>
-          <t>https://fairlac.iadb.org/estudio-dialogos-percepciones-de-futuro
-https://estudiodialogos.cl/</t>
+          <t>https://estudiodialogos.cl/
+https://fairlac.iadb.org/en/dialogos-study-perceptions-future</t>
         </is>
       </c>
       <c r="X15" s="2" t="inlineStr">
@@ -2464,8 +2464,8 @@
       </c>
       <c r="W16" s="2" t="inlineStr">
         <is>
-          <t>https://public.tableau.com/app/profile/ivania.yovanovic/viz/JornadasInstitutoPolticasPblicasUNAB/Dashboard3
-https://ipp.unab.cl/</t>
+          <t>https://ipp.unab.cl/
+https://public.tableau.com/app/profile/ivania.yovanovic/viz/JornadasInstitutoPolticasPblicasUNAB/Dashboard3</t>
         </is>
       </c>
       <c r="X16" s="2" t="inlineStr">
@@ -3977,8 +3977,7 @@
       </c>
       <c r="W29" s="2" t="inlineStr">
         <is>
-          <t>https://www.gobiernoabierto.ec/boletin-014-2023/
-https://ia.gobiernoabierto.ec/
+          <t>https://ia.gobiernoabierto.ec/
 https://ia.gobiernoabierto.ec/acercade</t>
         </is>
       </c>
@@ -4094,7 +4093,7 @@
       <c r="W30" s="2" t="inlineStr">
         <is>
           <t>https://dppa.medium.com/usando-el-poder-de-la-ia-para-impulsar-la-participaci%C3%B3n-pol%C3%ADtica-de-los-j%C3%B3venes-en-guatemala-6f6d7bf45a47
-https://www.fundaesq.org/guatemala-joven-la-voz-de-una-generacion-de-cambios/?utm_source=chatgpt.com
+https://www.fundaesq.org/guatemala-joven-la-voz-de-una-generacion-de-cambios/
 https://dppa.un.org/en/using-power-of-ai-to-boost-youth-political-participation-guatemala</t>
         </is>
       </c>
@@ -4777,9 +4776,9 @@
       </c>
       <c r="W36" s="2" t="inlineStr">
         <is>
-          <t>https://www.latinno.net/en/case/17232/
-https://www.gob.pe/institucion/cne/noticias/502734-lanzan-consulta-ciudadana-por-el-proyecto-educativo-nacional?utm_source=chatgpt.com
-https://cdn.www.gob.pe/uploads/document/file/1915017/CNE-%20proyecto-educativo-nacional-al-2036.pdf.pdf?v=1679434080</t>
+          <t>https://www.gob.pe/institucion/cne/noticias/502734-lanzan-consulta-ciudadana-por-el-proyecto-educativo-nacional
+https://cdn.www.gob.pe/uploads/document/file/1915017/CNE-%20proyecto-educativo-nacional-al-2036.pdf.pdf?v=1679434080
+https://andina.pe/agencia/noticia-usan-inteligencia-artificial-para-formular-proyecto-educativo-nacional-al-2036-777369.aspx</t>
         </is>
       </c>
       <c r="X36" s="2" t="inlineStr">
@@ -5450,8 +5449,8 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://participacion.digital.gob.cl/es-CL/folders/consultas-ciudadanas
-https://participacion.digital.gob.cl/projects/segunda-consulta-estrategia-de-gobierno-digital-2030</t>
+          <t>https://participacion.digital.gob.cl/projects/segunda-consulta-estrategia-de-gobierno-digital-2030
+https://participacion.digital.gob.cl/folders/consultas-ciudadanas</t>
         </is>
       </c>
     </row>
@@ -5563,8 +5562,8 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>https://public.tableau.com/app/profile/ivania.yovanovic/viz/JornadasInstitutoPolticasPblicasUNAB/Dashboard3
-https://ipp.unab.cl/</t>
+          <t>https://ipp.unab.cl/
+https://public.tableau.com/app/profile/ivania.yovanovic/viz/JornadasInstitutoPolticasPblicasUNAB/Dashboard3</t>
         </is>
       </c>
     </row>
@@ -6290,7 +6289,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/content/dam/oecd/es/publications/reports/2022/03/the-strategic-and-responsible-use-of-artificial-intelligence-in-the-public-sector-of-latin-america-and-the-caribbean_17c90e5e/5b189cb4-es.pdf#:~:text=Jaque%20y%20la%20Gu%C3%ADa%20de,Contiene%20informaci%C3%B3n%2C%20entre</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6586,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2303.15532?utm_source=chatgpt.com</t>
+          <t>https://arxiv.org/abs/2303.15532</t>
         </is>
       </c>
     </row>
@@ -6992,7 +6991,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://projects.itforchange.net/mavc/wp-content/uploads/2017/09/Voice-or-Chatter_Case-Study_Colombia_August-2017.pdf?utm_source=chatgpt.com</t>
+          <t>https://projects.itforchange.net/mavc/wp-content/uploads/2017/09/Voice-or-Chatter_Case-Study_Colombia_August-2017.pdf</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7180,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.undp.org/es/latin-america/comunicados-de-prensa/sara-la-nueva-herramienta-de-inteligencia-artificial-para-combatir-la-violencia-de-genero-en-centroamerica-0</t>
+          <t>https://www.undp.org/es/guatemala/comunicados-de-prensa/sara-la-nueva-herramienta-de-inteligencia-artificial-para-combatir-la-violencia-de-genero-en-centroamerica</t>
         </is>
       </c>
     </row>
@@ -7262,7 +7261,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.caf.com/es/actualidad/noticias/caf-realiza-su-primera-inversion-en-una-govtech-latinoamericana/</t>
+          <t>https://www.caf.com/es/actualidad/noticias/2021/07/caf-realiza-su-primera-inversion-en-una-govtech-latinoamericana/</t>
         </is>
       </c>
     </row>
@@ -7316,7 +7315,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.policylab.tech/post/revolucionando-la-denuncia-ciudadana-en-am%C3%A9rica-latina-con-tecnolog%C3%ADa-el-caso-del-chatbot-dci</t>
+          <t>https://www.policylab.tech/post/revolucionando-la-denuncia-ciudadana-en-am%C3%A9rica-latina-con-tecnolog%C3%ADa-el-caso-del-chatbot-dci-1</t>
         </is>
       </c>
     </row>
@@ -7559,7 +7558,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/content/dam/oecd/es/publications/reports/2022/03/the-strategic-and-responsible-use-of-artificial-intelligence-in-the-public-sector-of-latin-america-and-the-caribbean_17c90e5e/5b189cb4-es.pdf#:~:text=para%20identificar%20posibles%20trastornos,de%20las%20dificultades%20de%20%C3%ADndole</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7639,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>https://osf.io/cu6w3</t>
+          <t>https://algoritmoscide.org/proyectos/sufragio-seguro/</t>
         </is>
       </c>
     </row>
@@ -7694,7 +7693,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/content/dam/oecd/es/publications/reports/2022/03/the-strategic-and-responsible-use-of-artificial-intelligence-in-the-public-sector-of-latin-america-and-the-caribbean_17c90e5e/5b189cb4-es.pdf#:~:text=virtual%2Fchatbot%20que%20funciona%20por%20WhatsApp,que%20realice%20una%20observaci%C3%B3n%20f%C3%ADsica</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
     </row>
@@ -7802,7 +7801,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://fairlac.iadb.org/paraempleo</t>
+          <t>https://fairlac.iadb.org/en/paraempleo</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7828,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/content/dam/oecd/es/publications/reports/2022/03/the-strategic-and-responsible-use-of-artificial-intelligence-in-the-public-sector-of-latin-america-and-the-caribbean_17c90e5e/5b189cb4-es.pdf#:~:text=El%20chatbot%20virtual%20creado%20por,desarrollo%20de%20soluciones%20de%20IA</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
     </row>
@@ -7856,7 +7855,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.gub.uy/agencia-gobierno-electronico-sociedad-informacion-conocimiento/comunicacion/publicaciones/estrategia-nacional-inteligencia-artificial-2024-2030?utm_source=chatgpt.com</t>
+          <t>https://www.gub.uy/agencia-gobierno-electronico-sociedad-informacion-conocimiento/comunicacion/publicaciones/estrategia-nacional-inteligencia-artificial-2024-2030</t>
         </is>
       </c>
     </row>
@@ -8194,8 +8193,8 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2511.01545
-https://arxiv.org/abs/2509.21292
+          <t>https://arxiv.org/abs/2509.21292
+https://arxiv.org/abs/2511.01545
 https://github.com/ResidenciaTICBrisa/BP-Classificador-de-Propostas
 https://www.gov.br/secretariageral/pt-br/noticias/2024/dezembro/secretaria-geral-da-presidencia-formaliza-parceria-com-plataforma-decidim
 https://www.gov.br/secretariageral/pt-br/noticias/2025/novembro/brasil-participativo-integra-comite-internacional-de-democracia-digital
@@ -8704,7 +8703,7 @@
         <is>
           <t>https://www.bcn.cl/procesoconstituyente/cabildos2016/
 https://aclanthology.org/W17-5101/
-https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0267443</t>
+https://journals.plos.org/plosone/article?id=10.1371%2Fjournal.pone.0267443</t>
         </is>
       </c>
     </row>
@@ -8834,8 +8833,8 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>https://participacion.digital.gob.cl/es-CL/folders/consultas-ciudadanas
-https://participacion.digital.gob.cl/projects/segunda-consulta-estrategia-de-gobierno-digital-2030</t>
+          <t>https://participacion.digital.gob.cl/projects/segunda-consulta-estrategia-de-gobierno-digital-2030
+https://participacion.digital.gob.cl/folders/consultas-ciudadanas</t>
         </is>
       </c>
     </row>
@@ -8897,8 +8896,8 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>https://fairlac.iadb.org/estudio-dialogos-percepciones-de-futuro
-https://estudiodialogos.cl/</t>
+          <t>https://estudiodialogos.cl/
+https://fairlac.iadb.org/en/dialogos-study-perceptions-future</t>
         </is>
       </c>
     </row>
@@ -8960,8 +8959,8 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>https://public.tableau.com/app/profile/ivania.yovanovic/viz/JornadasInstitutoPolticasPblicasUNAB/Dashboard3
-https://ipp.unab.cl/</t>
+          <t>https://ipp.unab.cl/
+https://public.tableau.com/app/profile/ivania.yovanovic/viz/JornadasInstitutoPolticasPblicasUNAB/Dashboard3</t>
         </is>
       </c>
     </row>
@@ -9370,8 +9369,8 @@
       <c r="K23" s="12" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>https://www.govocal.com/
-https://vinadecide.cl/pages/presupuestoparticipativo</t>
+          <t>https://vinadecide.cl/pages/presupuestoparticipativo
+https://www.govocal.com/</t>
         </is>
       </c>
     </row>
@@ -9746,7 +9745,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>https://www.gobiernoabierto.ec/boletin-014-2023/
+          <t>https://ia.gobiernoabierto.ec/
 https://ia.gobiernoabierto.ec/
 https://ia.gobiernoabierto.ec/acercade</t>
         </is>
@@ -9811,7 +9810,7 @@
       <c r="L30" s="2" t="inlineStr">
         <is>
           <t>https://dppa.medium.com/usando-el-poder-de-la-ia-para-impulsar-la-participaci%C3%B3n-pol%C3%ADtica-de-los-j%C3%B3venes-en-guatemala-6f6d7bf45a47
-https://www.fundaesq.org/guatemala-joven-la-voz-de-una-generacion-de-cambios/?utm_source=chatgpt.com
+https://www.fundaesq.org/guatemala-joven-la-voz-de-una-generacion-de-cambios/
 https://dppa.un.org/en/using-power-of-ai-to-boost-youth-political-participation-guatemala</t>
         </is>
       </c>
@@ -10191,8 +10190,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>https://www.latinno.net/en/case/17232/
-https://www.gob.pe/institucion/cne/noticias/502734-lanzan-consulta-ciudadana-por-el-proyecto-educativo-nacional?utm_source=chatgpt.com
+          <t>https://www.gob.pe/institucion/cne/noticias/502734-lanzan-consulta-ciudadana-por-el-proyecto-educativo-nacional
 https://cdn.www.gob.pe/uploads/document/file/1915017/CNE-%20proyecto-educativo-nacional-al-2036.pdf.pdf?v=1679434080
 https://andina.pe/agencia/noticia-usan-inteligencia-artificial-para-formular-proyecto-educativo-nacional-al-2036-777369.aspx
 https://elperuano.pe/noticia/87397-usan-inteligencia-artificial-para-formular-el-proyecto-educativo-nacional-al-2036</t>

</xml_diff>

<commit_message>
Reincorporar CU Código de las Familias (SÍ); UCampus revisado se mantiene NO
Confirmación web de los 2 posibles reingresos:
- CU Consulta Popular Código de las Familias → SÍ. GEMA-CEN (Datys) procesa el
  contenido de las propuestas: recuperación de información + agrupamiento por
  similitud textual + clasificación por temas ('propuestas típicas'), con
  validación de juristas. Fuentes: ficha Datys + Granma.
- CL UCampus → se mantiene NO. Fue el operador tecnológico (recepción/gestión);
  la sistematización de sus mecanismos fue cualitativa por académicos. El NLP
  sobre aportes (IMFD+PUC, Consulta Ciudadana) ya está capturado en el caso
  'Participación Ciudadana Proceso Constitucional'.

Lista de posibles reingresos vaciada (ambos resueltos). Sin DUDAs pendientes.
Estado final: 35 SÍ · 0 DUDA · 72 NO → 34 iniciativas efectivas.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/planilla_ILIA2026_SIMPLE.xlsx
+++ b/data/gates/planilla_ILIA2026_SIMPLE.xlsx
@@ -15,10 +15,10 @@
     <sheet name="6 · Metodología (CENIA v2)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 · Casos (entran+dudosos)'!$A$1:$X$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 · A validar a mano'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3 · Excluidos'!$A$1:$E$74</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4 · Evidencia y fuentes'!$A$1:$L$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 · Casos (entran+dudosos)'!$A$1:$X$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 · A validar a mano'!$A$1:$G$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3 · Excluidos'!$A$1:$E$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4 · Evidencia y fuentes'!$A$1:$L$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -582,7 +582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X35"/>
+  <dimension ref="A1:X36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3641,12 +3641,12 @@
       <c r="A27" s="2" t="inlineStr"/>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>CU</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAGA IA </t>
+          <t>Consulta Popular Código de las Familias (GEMA-CEN / XISCOP)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -3666,17 +3666,17 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>ALTA (baseline 2025 + reverif. web 2026)</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Referendos e Iniciativas Populares</t>
+          <t>Participación Digital; Referendos e Iniciativas Populares</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="J27" s="2" t="n">
@@ -3684,17 +3684,17 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Plataforma</t>
+          <t>Uso único</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>gobierno nacional; sociedad civil</t>
+          <t>gobierno nacional</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Mixto</t>
+          <t>Público</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil</t>
+          <t>Privado; Academia; Gobierno</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3714,41 +3714,42 @@
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>LLM</t>
+          <t>NLP; Minería de texto; Recuperación de información; Clasificación automática de documentos</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>Plataforma que utiliza inteligencia artificial para asistir en la creación de compromisos de Estado Abierto. Analiza datos de planes de acción de gobierno abierto de Ecuador y otros países de Hispanoamérica para sugerir actividades e hitos relacionados con temas propuestos por los usuarios</t>
+          <t>Consulta popular legislativa nacional sobre el proyecto del Código de las Familias en Cuba, organizada y supervisada por el Consejo Electoral Nacional (CEN). Se desarrolló entre febrero y abril de 2022 mediante más de 79.000 reuniones en barrios, centros laborales y estudiantiles, con la participación de unos 6.481.200 personas que emitieron opiniones y propuestas sobre el articulado del proyecto de ley. Las propuestas recogidas eran revisadas y clasificadas por juristas en el sistema XISCOP y luego procesadas en el sistema GEMA-CEN, que mediante 'análisis inteligente de los expedientes' agrupaba propuestas similares y determinaba 'propuestas típicas' por párrafo/categoría (se determinaron 5.237 propuestas típicas por Título). XISCOP (UCI) emitía además las estadísticas oficiales. El proceso de consulta cerró en abril de 2022; el Código fue aprobado posteriormente en referendo el 25 de septiembre de 2022.</t>
         </is>
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t>Gobierno Abierto Ecuador, en colaboración con la Fundación de Ayuda por Internet (Fundapi)</t>
+          <t>Consejo Electoral Nacional (CEN) de Cuba como órgano organizador y supervisor de la consulta popular. El procesamiento informático se apoyó en dos sistemas: XISCOP, desarrollado por la Universidad de las Ciencias Informáticas (UCI), para la entrada, revisión, clasificación y estadísticas oficiales; y GEMA-CEN, basado en el producto GEMA de la empresa estatal Datys, para el 'análisis inteligente' y agrupamiento de las propuestas. La Asamblea Nacional del Poder Popular y la Comisión redactora del Ministerio de Justicia recibieron los resultados.</t>
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="V27" s="4" t="n">
-        <v>0</v>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="V27" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="W27" s="2" t="inlineStr">
         <is>
-          <t>https://ia.gobiernoabierto.ec/
-https://ia.gobiernoabierto.ec/acercade</t>
+          <t>http://www.datys.cu/spa/site/product/15
+https://www.granma.cu/cuba/2022-01-24/herramientas-digitales-seran-claves-durante-la-consulta-popular-del-codigo-de-las-familias-24-01-2022-13-01-18
+https://www.uci.cu/</t>
         </is>
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>EC-paga-ia</t>
+          <t>CU-consulta-popular-codigo-de-las-familias</t>
         </is>
       </c>
     </row>
@@ -3756,12 +3757,12 @@
       <c r="A28" s="2" t="inlineStr"/>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guatemala Joven Conversa </t>
+          <t xml:space="preserve">PAGA IA </t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -3786,7 +3787,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
+          <t>Referendos e Iniciativas Populares</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -3799,12 +3800,12 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Uso único</t>
+          <t>Plataforma</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>organización internacional; sociedad civil</t>
+          <t>gobierno nacional; sociedad civil</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -3819,208 +3820,209 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>Gobierno</t>
+          <t>Sociedad Civil</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>NLP - Sentiment; NLP - Tópicos</t>
+          <t>LLM</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>Iniciativa de diálogos digitales asistidos por inteligencia artificial que reunió a más de 300 jóvenes de los 22 departamentos de Guatemala para discutir temas como la reforma electoral, la participación juvenil en el desarrollo y la lucha contra la corrupción.</t>
+          <t>Plataforma que utiliza inteligencia artificial para asistir en la creación de compromisos de Estado Abierto. Analiza datos de planes de acción de gobierno abierto de Ecuador y otros países de Hispanoamérica para sugerir actividades e hitos relacionados con temas propuestos por los usuarios</t>
         </is>
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
-          <t>Oficina del Coordinador Residente de las Naciones Unidas en Guatemala y Fundación Esquipulas para la Paz, la Democracia, el Desarrollo y la Integración</t>
+          <t>Gobierno Abierto Ecuador, en colaboración con la Fundación de Ayuda por Internet (Fundapi)</t>
         </is>
       </c>
       <c r="U28" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="V28" s="4" t="n">
         <v>0</v>
       </c>
       <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t>https://ia.gobiernoabierto.ec/
+https://ia.gobiernoabierto.ec/acercade</t>
+        </is>
+      </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>EC-paga-ia</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>GT</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Guatemala Joven Conversa </t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>ALTA (baseline 2025 + reverif. web 2026)</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Gobernanza Colaborativa</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Implementación</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Uso único</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>organización internacional; sociedad civil</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Mixto</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>contenido</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>Gobierno</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>NLP - Sentiment; NLP - Tópicos</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>Iniciativa de diálogos digitales asistidos por inteligencia artificial que reunió a más de 300 jóvenes de los 22 departamentos de Guatemala para discutir temas como la reforma electoral, la participación juvenil en el desarrollo y la lucha contra la corrupción.</t>
+        </is>
+      </c>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>Oficina del Coordinador Residente de las Naciones Unidas en Guatemala y Fundación Esquipulas para la Paz, la Democracia, el Desarrollo y la Integración</t>
+        </is>
+      </c>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="V29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W29" s="2" t="inlineStr">
         <is>
           <t>https://dppa.medium.com/usando-el-poder-de-la-ia-para-impulsar-la-participaci%C3%B3n-pol%C3%ADtica-de-los-j%C3%B3venes-en-guatemala-6f6d7bf45a47
 https://www.fundaesq.org/guatemala-joven-la-voz-de-una-generacion-de-cambios/
 https://dppa.un.org/en/using-power-of-ai-to-boost-youth-political-participation-guatemala</t>
         </is>
       </c>
-      <c r="X28" s="2" t="inlineStr">
+      <c r="X29" s="2" t="inlineStr">
         <is>
           <t>GT-guatemala-joven-conversa</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>➜ RESCATADO → ENTRA (criterio corregido)</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>HN</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">RedPública + iVerify </t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>ALTA (baseline 2025 + reverif. web 2026)</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Referendos e Iniciativas Populares</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>Análisis</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>Uso único</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>organización internacional; universidad</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>Público</t>
-        </is>
-      </c>
-      <c r="N29" s="2" t="inlineStr">
-        <is>
-          <t>contenido</t>
-        </is>
-      </c>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>Gobierno; Academia</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="inlineStr">
-        <is>
-          <t>Internacional, Nacional</t>
-        </is>
-      </c>
-      <c r="Q29" s="2" t="inlineStr">
-        <is>
-          <t>NLP - Tópicos</t>
-        </is>
-      </c>
-      <c r="R29" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S29" s="2" t="inlineStr">
-        <is>
-          <t>Plataforma digital que recibe propuestas de ley y proyectos sociales, con un módulo de análisis que agrupa temas y genera tableros de tendencias. Integra iVerify, una herramienta que utiliza aprendizaje automático para detectar y clasificar desinformación electoral antes de su publicación.</t>
-        </is>
-      </c>
-      <c r="T29" s="2" t="inlineStr">
-        <is>
-          <t>Programa de las Naciones Unidas para el Desarrollo (PNUD) en colaboración con CEUTEC y la Unión Europea.</t>
-        </is>
-      </c>
-      <c r="U29" s="2" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="V29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.undp.org/es/honduras/historias/participacion-ciudadana-con-innovacion-digital-traves-de-redpublica-honduras</t>
-        </is>
-      </c>
-      <c r="X29" s="2" t="inlineStr">
-        <is>
-          <t>HN-redpublica-iverify</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>Gobernanza Colaborativa; Participación Digital</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -4038,228 +4040,228 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
+          <t>organización internacional; universidad</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Público</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>contenido</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Gobierno; Academia</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>Internacional, Nacional</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>NLP - Tópicos</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S30" s="2" t="inlineStr">
+        <is>
+          <t>Plataforma digital que recibe propuestas de ley y proyectos sociales, con un módulo de análisis que agrupa temas y genera tableros de tendencias. Integra iVerify, una herramienta que utiliza aprendizaje automático para detectar y clasificar desinformación electoral antes de su publicación.</t>
+        </is>
+      </c>
+      <c r="T30" s="2" t="inlineStr">
+        <is>
+          <t>Programa de las Naciones Unidas para el Desarrollo (PNUD) en colaboración con CEUTEC y la Unión Europea.</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="V30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/es/honduras/historias/participacion-ciudadana-con-innovacion-digital-traves-de-redpublica-honduras</t>
+        </is>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>HN-redpublica-iverify</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Gobernanza Colaborativa; Participación Digital</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Análisis</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Uso único</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
           <t>gobierno local</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>Público</t>
         </is>
       </c>
-      <c r="N30" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>contenido</t>
         </is>
       </c>
-      <c r="O30" s="2" t="inlineStr">
+      <c r="O31" s="2" t="inlineStr">
         <is>
           <t>Gobierno</t>
         </is>
       </c>
-      <c r="P30" s="2" t="inlineStr">
+      <c r="P31" s="2" t="inlineStr">
         <is>
           <t>Nacional</t>
         </is>
       </c>
-      <c r="Q30" s="2" t="inlineStr">
+      <c r="Q31" s="2" t="inlineStr">
         <is>
           <t>NLP; Otros(no especificado)</t>
         </is>
       </c>
-      <c r="R30" s="2" t="inlineStr">
+      <c r="R31" s="2" t="inlineStr">
         <is>
           <t>no-claro</t>
         </is>
       </c>
-      <c r="S30" s="2" t="inlineStr">
+      <c r="S31" s="2" t="inlineStr">
         <is>
           <t>Elaboración del Programa de Gobierno del Estado de Guanajuato 2024-2030 ('Gobierno de la Gente'), un plan de gobierno construido con participación ciudadana: se recorrió el territorio y se realizaron cuatro talleres regionales (noreste, norte, centro y sur) con representación de los 46 municipios, integrando la voz de más de 26,000 personas mediante talleres y consultas. El contenido fue validado por el Consejo de Planeación para el Desarrollo del Estado de Guanajuato (COPLADEG), conformado por ciudadanía, la Gobernadora, secretarios de cada eje e IPLANEG. Se utilizaron herramientas de inteligencia artificial para procesar y organizar las miles de ideas y propuestas recibidas, identificar las prioridades más mencionadas por la ciudadanía y entender las necesidades de cada región, transformando el diálogo social en datos para la toma de decisiones que alimentaron los ejes del programa. Adicionalmente existe la asistente virtual 'Esperanza' para consultar el programa ya publicado.</t>
         </is>
       </c>
-      <c r="T30" s="2" t="inlineStr">
+      <c r="T31" s="2" t="inlineStr">
         <is>
           <t>Gobierno del Estado de Guanajuato — Instituto de Planeación, Estadística y Geografía del Estado de Guanajuato (IPLANEG), con validación del COPLADEG. Titular: Gobernadora Libia Dennise García Muñoz Ledo.</t>
         </is>
       </c>
-      <c r="U30" s="2" t="inlineStr">
+      <c r="U31" s="2" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="V30" s="5" t="n">
+      <c r="V31" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="W30" s="2" t="inlineStr">
+      <c r="W31" s="2" t="inlineStr">
         <is>
           <t>https://guanajuatointeligente.com/como-hicimos-el-programa/
 https://iplaneg.guanajuato.gob.mx/programagobierno24-30/
 https://iplaneg.guanajuato.gob.mx/wp-content/uploads/03-2.05-Diagnostico-Programa-de-Gobierno-2024-2030-_Diagnostico-Estatal-2025_.pdf</t>
         </is>
       </c>
-      <c r="X30" s="2" t="inlineStr">
+      <c r="X31" s="2" t="inlineStr">
         <is>
           <t>MX-guanajuato-inteligente-2024-2030</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>➜ RESCATADO → ENTRA (criterio corregido)</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Presupuesto CRECES</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>MEDIA (baseline 2025; sin señal web 2026 nueva)</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Presupuestos Participativos</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Implementación</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Uso único</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>gobierno local</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>Público</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>contenido</t>
-        </is>
-      </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>Privado</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="Q31" s="2" t="inlineStr">
-        <is>
-          <t>Chatbot - Inespecífico</t>
-        </is>
-      </c>
-      <c r="R31" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S31" s="2" t="inlineStr">
-        <is>
-          <t>Presupuesto participativo del Ayuntamiento de Hermosillo en México. Utiliza un chatbot que a través de IA simplifica y facilita la votación de los presupuestos participativos</t>
-        </is>
-      </c>
-      <c r="T31" s="2" t="inlineStr">
-        <is>
-          <t>Ayundamiento de Hermosilla</t>
-        </is>
-      </c>
-      <c r="U31" s="2" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="V31" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="W31" s="2" t="inlineStr">
-        <is>
-          <t>https://presupuestocreces.hermosillo.gob.mx/</t>
-        </is>
-      </c>
-      <c r="X31" s="2" t="inlineStr">
-        <is>
-          <t>MX-presupuesto-creces</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Participación Digital; Gobernanza Colaborativa</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Análisis; Traducción Política</t>
         </is>
       </c>
       <c r="J32" s="2" t="n">
@@ -4267,419 +4269,533 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
+          <t>Uso único</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>gobierno local</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Público</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>contenido</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>Chatbot - Inespecífico</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>Presupuesto participativo del Ayuntamiento de Hermosillo en México. Utiliza un chatbot que a través de IA simplifica y facilita la votación de los presupuestos participativos</t>
+        </is>
+      </c>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>Ayundamiento de Hermosilla</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="V32" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t>https://presupuestocreces.hermosillo.gob.mx/</t>
+        </is>
+      </c>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>MX-presupuesto-creces</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Participación Digital; Gobernanza Colaborativa</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Análisis; Traducción Política</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
           <t>Plataforma</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>sociedad civil; gobierno nacional</t>
         </is>
       </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>Privado</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>contenido</t>
         </is>
       </c>
-      <c r="O32" s="2" t="inlineStr">
+      <c r="O33" s="2" t="inlineStr">
         <is>
           <t>Sociedad Civil</t>
         </is>
       </c>
-      <c r="P32" s="2" t="inlineStr">
+      <c r="P33" s="2" t="inlineStr">
         <is>
           <t>Nacional</t>
         </is>
       </c>
-      <c r="Q32" s="2" t="inlineStr"/>
-      <c r="R32" s="2" t="inlineStr">
+      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr">
         <is>
           <t>no-claro</t>
         </is>
       </c>
-      <c r="S32" s="2" t="inlineStr">
+      <c r="S33" s="2" t="inlineStr">
         <is>
           <t>Mansa Idea (www.mansaidea.com) es una plataforma digital basada en inteligencia artificial lanzada el 1 de abril de 2024 por la Fundación Panamá Participa (sociedad civil), liderada por Paulina Franceschi. La plataforma organiza y hace navegables más de 175.000 ideas y propuestas ciudadanas generadas durante el Pacto del Bicentenario 'Cerrando Brechas' (proceso participativo nacional convocado por el gobierno de Panamá / Concertación Nacional, presidente Cortizo, 2020-2021), agregando los consensos nacionales y regionales/provinciales por tema en un solo clic. La IA se aplica sobre el CONTENIDO de los aportes ciudadanos (organiza, agrega y sintetiza el corpus de propuestas) para convertirlo en una base de datos navegable. El uso de la IA es un tratamiento PUNTERAL (~2024) de un corpus histórico de un proceso participativo ya cerrado (el Pacto fue 2020-2021), orientado a elevar el nivel de la conversación electoral 2024 y a dotar a candidatos, medios y ciudadanía de una herramienta para alinear planes con las necesidades de la población y monitorear el mandato ciudadano. IMPORTANTE: el proceso participativo original (recolección de aportes) fue convocado por el gobierno; la capa de IA (Mansa Idea) la desarrolla la sociedad civil sobre ese corpus ya recolectado.</t>
         </is>
       </c>
-      <c r="T32" s="2" t="inlineStr">
+      <c r="T33" s="2" t="inlineStr">
         <is>
           <t>Fundación Panamá Participa (sociedad civil, Panamá), iniciativa liderada por Paulina Franceschi. El proceso participativo de origen (Pacto del Bicentenario 'Cerrando Brechas') fue convocado por el Gobierno de Panamá a través del mecanismo de Concertación Nacional para el Desarrollo (presidente Laurentino Cortizo), con apoyo del PNUD.</t>
         </is>
       </c>
-      <c r="U32" s="2" t="inlineStr">
+      <c r="U33" s="2" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="V32" s="5" t="n">
+      <c r="V33" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="W32" s="2" t="inlineStr">
+      <c r="W33" s="2" t="inlineStr">
         <is>
           <t>https://mansaidea.com/ (intentar archive.org / cache); buscar 'Mansa Idea metodología inteligencia artificial procesamiento propuestas' y entrevistas técnicas a Paulina Franceschi / Fundación Panamá Participa.
 https://mansaidea.com/ ; buscar 'Mansa Idea 2025' / 'Mansa Idea 2026' / 'Fundación Panamá Participa actividad reciente'.
 https://mansaidea.com/ ; buscar evidencia de actualizaciones periódicas del corpus o nuevas convocatorias.</t>
         </is>
       </c>
-      <c r="X32" s="2" t="inlineStr">
+      <c r="X33" s="2" t="inlineStr">
         <is>
           <t>PA-mansa-idea-pacto-del-bicentenario</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr"/>
-      <c r="B33" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>PE</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>ALTA (baseline 2025 + reverif. web 2026)</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Gobernanza Colaborativa</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>Análisis</t>
         </is>
       </c>
-      <c r="J33" s="2" t="n">
+      <c r="J34" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Uso único</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>otra institución pública</t>
         </is>
       </c>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>Público</t>
         </is>
       </c>
-      <c r="N33" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>contenido</t>
         </is>
       </c>
-      <c r="O33" s="2" t="inlineStr">
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>Privado</t>
         </is>
       </c>
-      <c r="P33" s="2" t="inlineStr">
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>Internacional</t>
         </is>
       </c>
-      <c r="Q33" s="2" t="inlineStr">
+      <c r="Q34" s="2" t="inlineStr">
         <is>
           <t>NLP - Tópicos; NLP - Sentiment</t>
         </is>
       </c>
-      <c r="R33" s="2" t="inlineStr">
+      <c r="R34" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="S33" s="2" t="inlineStr">
+      <c r="S34" s="2" t="inlineStr">
         <is>
           <t>Una consulta pública para recoger opiniones sobre el Proyecto Educativo Nacional 2036, utilizando encuestas en línea, talleres y mesas deliberativas.</t>
         </is>
       </c>
-      <c r="T33" s="2" t="inlineStr">
+      <c r="T34" s="2" t="inlineStr">
         <is>
           <t>Consejo Nacional de Educación del Perú</t>
         </is>
       </c>
-      <c r="U33" s="2" t="inlineStr">
+      <c r="U34" s="2" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="V33" s="4" t="n">
+      <c r="V34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W33" s="2" t="inlineStr">
+      <c r="W34" s="2" t="inlineStr">
         <is>
           <t>https://www.gob.pe/institucion/cne/noticias/502734-lanzan-consulta-ciudadana-por-el-proyecto-educativo-nacional
 https://cdn.www.gob.pe/uploads/document/file/1915017/CNE-%20proyecto-educativo-nacional-al-2036.pdf.pdf?v=1679434080
 https://andina.pe/agencia/noticia-usan-inteligencia-artificial-para-formular-proyecto-educativo-nacional-al-2036-777369.aspx</t>
         </is>
       </c>
-      <c r="X33" s="2" t="inlineStr">
+      <c r="X34" s="2" t="inlineStr">
         <is>
           <t>PE-consulta-ciudadana-sobre-el-proyecto-nac</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>➜ RESCATADO → ENTRA (criterio corregido)</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>TT</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr">
         <is>
           <t>DUDA(lean NO)</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Participación Digital; Gobernanza Colaborativa</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="n">
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Plataforma</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>gobierno nacional</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>Público</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>no-claro</t>
         </is>
       </c>
-      <c r="O34" s="2" t="inlineStr">
+      <c r="O35" s="2" t="inlineStr">
         <is>
           <t>Privado</t>
         </is>
       </c>
-      <c r="P34" s="2" t="inlineStr">
+      <c r="P35" s="2" t="inlineStr">
         <is>
           <t>Internacional</t>
         </is>
       </c>
-      <c r="Q34" s="2" t="inlineStr">
+      <c r="Q35" s="2" t="inlineStr">
         <is>
           <t>NLP; Resumen automatico; Clasificacion/agrupacion de texto (capacidad de la plataforma sujeta a plan Premium; activacion NO confirmada en TT)</t>
         </is>
       </c>
-      <c r="R34" s="2" t="inlineStr">
+      <c r="R35" s="2" t="inlineStr">
         <is>
           <t>no-claro</t>
         </is>
       </c>
-      <c r="S34" s="2" t="inlineStr">
+      <c r="S35" s="2" t="inlineStr">
         <is>
           <t>EngageTT (engage.gov.tt) es la plataforma de participacion ciudadana del Ministry of Digital Transformation de Trinidad y Tobago (desde mayo 2025 fusionado en el Ministry of Public Administration and Artificial Intelligence, MPAAI), lanzada en el simposio del NDTS el 12 de febrero de 2025 junto al BID (IDB). Se usa como canal de participacion en el proceso de planificacion nacional del National Digital Transformation Strategy (NDTS) 2024-2027, donde ciudadanos, empresas y partes interesadas reciben actualizaciones y aportan retroalimentacion via encuestas, sondeos (polls), un 'Open Forum' de ideas y el envio de propuestas. La instancia corre sobre el software Go Vocal (antes CitizenLab) -confirmado por la ruta interna 'projects/e-democracy-govocal-internal'-. Go Vocal incorpora un modulo de IA/NLP de 'Sensemaking' (analisis y resumen automatico de aportes), pero ese modulo NO viene activo por defecto: segun la documentacion de soporte de Go Vocal, el acceso a la funcion de AI Analysis/Sensemaking DEPENDE DEL PLAN contratado (Advanced Sensemaking con auto-insights esta en el plan Premium). Tras 2a pasada de investigacion (&gt;=14 busquedas/fetches) NO se halla evidencia alguna de que la instancia de Trinidad active ni use esas funciones de IA sobre el CONTENIDO de los aportes; toda la documentacion describe a EngageTT como recolector (surveys, polls, Open Forum, ideas), es decir plataforma usada como formulario sin analisis automatico confirmado. Existe ademas AskNDTS, un chatbot/PWA de IA conversacional para responder preguntas sobre el NDTS (rol de FAQ informativo, EXCLUIDO del criterio).</t>
         </is>
       </c>
-      <c r="T34" s="2" t="inlineStr">
+      <c r="T35" s="2" t="inlineStr">
         <is>
           <t>Ministry of Digital Transformation de Trinidad y Tobago (desde el 23-may-2025 fusionado en el Ministry of Public Administration and Artificial Intelligence, MPAAI), en colaboracion con el Banco Interamericano de Desarrollo (BID/IDB). Plataforma de software: Go Vocal (antes CitizenLab), empresa belga.</t>
         </is>
       </c>
-      <c r="U34" s="2" t="inlineStr">
+      <c r="U35" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="V34" s="5" t="n">
+      <c r="V35" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="W34" s="2" t="inlineStr">
+      <c r="W35" s="2" t="inlineStr">
         <is>
           <t>https://engage.gov.tt/ideas/ndts-2025-actionable-feedback-implementation-plan
 https://www.govocal.com/plans
 https://support.govocal.com/en/articles/9015305-faq-on-our-ai-sensemaking-tool</t>
         </is>
       </c>
-      <c r="X34" s="2" t="inlineStr">
+      <c r="X35" s="2" t="inlineStr">
         <is>
           <t>TT-engagett-plataforma-go-vocal</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
-      <c r="B35" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr"/>
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>UY</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Pol.is en el Referéndum Nacional de la LUC (Uruguay) — equipo UdelaR</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>(sin revisar)</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>MEDIA (fuente primaria + OCDE 2025; fetch primario bloqueado por proxy, citas vía repo/WebSearch)</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Referendos e Iniciativas Populares</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>Análisis</t>
         </is>
       </c>
-      <c r="J35" s="2" t="n">
+      <c r="J36" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Uso único</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>universidad</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>Público</t>
         </is>
       </c>
-      <c r="N35" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr">
         <is>
           <t>contenido</t>
         </is>
       </c>
-      <c r="O35" s="2" t="inlineStr">
+      <c r="O36" s="2" t="inlineStr">
         <is>
           <t>Sociedad Civil; Academia</t>
         </is>
       </c>
-      <c r="P35" s="2" t="inlineStr">
+      <c r="P36" s="2" t="inlineStr">
         <is>
           <t>Internacional</t>
         </is>
       </c>
-      <c r="Q35" s="2" t="inlineStr">
+      <c r="Q36" s="2" t="inlineStr">
         <is>
           <t>Clustering; ML - Inespecífico</t>
         </is>
       </c>
-      <c r="R35" s="2" t="inlineStr">
+      <c r="R36" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="S35" s="2" t="inlineStr">
+      <c r="S36" s="2" t="inlineStr">
         <is>
           <t>Referéndum nacional para derogar 135 artículos de la Ley de Urgente Consideración (LUC). Un equipo de la Universidad de la República corrió una conversación Pol.is en paralelo al referéndum del 27/03/2022 (documentado como caso 2021).</t>
         </is>
       </c>
-      <c r="T35" s="2" t="inlineStr">
+      <c r="T36" s="2" t="inlineStr">
         <is>
           <t>Equipo de 13 personas de la Universidad de la República (UdelaR) — ingenieros, comunicadores y científicos de datos; plataforma Pol.is (The Computational Democracy Project)</t>
         </is>
       </c>
-      <c r="U35" s="2" t="inlineStr">
+      <c r="U36" s="2" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="V35" s="5" t="n">
+      <c r="V36" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="W35" s="2" t="inlineStr">
+      <c r="W36" s="2" t="inlineStr">
         <is>
           <t>https://compdemocracy.org/case-studies/2021-uruguay-national-referendum/</t>
         </is>
       </c>
-      <c r="X35" s="2" t="inlineStr">
+      <c r="X36" s="2" t="inlineStr">
         <is>
           <t>UY-polis-referendum-luc</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X35"/>
+  <autoFilter ref="A1:X36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4690,7 +4806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5494,149 +5610,73 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>F. Posible reingreso</t>
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>G. Dedup (confirmar)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>¿Reingresa? (SI/NO)</t>
+          <t>Confirmar cuenta como 1</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>e-Cidadania (Senado Federal)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>El 'matching de ideias' no se cuenta aparte del 'marcado de audiencias' (misma plataforma)</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>'Duas ferramentas relacionadas' del mismo portal e-Cidadania (fuente Senado).</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>G. Dedup (confirmar)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Confirmar 1 SI + 1 NO</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Plataforma UCampus - participación 2023 (proceso constitucional)</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Verificar si corresponde reingresarlo</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Su referencia lo marca RESCATABLE (confirmar si hubo NLP sobre los aportes del proceso constituyente).</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>https://ingenieria.uchile.cl/noticias/204877/-participacion-ciudadana-proceso-constitucional-sera-por-ucampus
-https://www.secretariadeparticipacion.cl/wp-content/uploads/2023/10/Informe-SPC-Final.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>F. Posible reingreso</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>¿Reingresa? (SI/NO)</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>CU</t>
-        </is>
-      </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Consulta Popular Código de las Familias (GEMA-CEN / XISCOP)</t>
+          <t>Participación Ciudadana Proceso Constitucional</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Verificar si corresponde reingresarlo</t>
+          <t>Homónimo duplicado: uno cuenta (SI), el otro NO</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Su referencia lo marca RESCATABLE; mi evidencia (ficha técnica Datys/GEMA = NLP) apoya SI.</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>http://www.datys.cu/spa/site/product/15
-https://www.granma.cu/cuba/2022-01-24/herramientas-digitales-seran-claves-durante-la-consulta-popular-del-codigo-de-las-familias-24-01-2022-13-01-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>G. Dedup (confirmar)</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Confirmar cuenta como 1</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>BR</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>e-Cidadania (Senado Federal)</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>El 'matching de ideias' no se cuenta aparte del 'marcado de audiencias' (misma plataforma)</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>'Duas ferramentas relacionadas' del mismo portal e-Cidadania (fuente Senado).</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>G. Dedup (confirmar)</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Confirmar 1 SI + 1 NO</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Participación Ciudadana Proceso Constitucional</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Homónimo duplicado: uno cuenta (SI), el otro NO</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
           <t>Ya resuelto en la planilla.</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G25"/>
+  <autoFilter ref="A1:G23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5647,7 +5687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6821,27 +6861,27 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>CU</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Consulta Popular Código de las Familias (GEMA-CEN / XISCOP)</t>
+          <t>CiudadanIA</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Dudoso</t>
+          <t>Excluido (criterio corregido)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Dentro de un proceso participativo formal y de gran escala (consulta popular legislativa nacional sobre el Código de las Familias, feb-abr 2022, ~6,5 millones de participantes y cientos de miles de propuestas) se usó IA sobre el CONTENIDO de los aportes ciudadanos: el sistema GEMA-CEN (basado en GEM</t>
+          <t>Solo atención/servicio; la 'participación' es co-diseñar la IA aportando datos, no consulta pública. Sin módulo de participación (verificado). Decisión del equipo.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>http://www.datys.cu/spa/site/product/15</t>
+          <t>https://www.genia.ai/paises-miembros</t>
         </is>
       </c>
     </row>
@@ -6853,22 +6893,22 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>CiudadanIA</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Excluido (criterio corregido)</t>
+          <t>Excluido 2025</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Solo atención/servicio; la 'participación' es co-diseñar la IA aportando datos, no consulta pública. Sin módulo de participación (verificado). Decisión del equipo.</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.genia.ai/paises-miembros</t>
+          <t>https://www.undp.org/es/guatemala/comunicados-de-prensa/sara-la-nueva-herramienta-de-inteligencia-artificial-para-combatir-la-violencia-de-genero-en-centroamerica</t>
         </is>
       </c>
     </row>
@@ -6880,7 +6920,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>TAÍNA: Gobierno Inteligente</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -6890,66 +6930,66 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>Atención ciudadana</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.undp.org/es/guatemala/comunicados-de-prensa/sara-la-nueva-herramienta-de-inteligencia-artificial-para-combatir-la-violencia-de-genero-en-centroamerica</t>
+          <t>https://www.diariolibre.com/actualidad/nacional/2023/10/11/gobierno-presenta-estrategia-de-inteligencia-artificial/2489157</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>TAÍNA: Gobierno Inteligente</t>
+          <t>Plataforma de modelos generativos de IA de SEGEPLAN + Red Ciudadana (Guatemala)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Excluido 2025</t>
+          <t>Descubrimiento</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Atención ciudadana</t>
+          <t>El criterio ELEGIBLE exige que la IA generativa se use para SISTEMATIZAR/CLASIFICAR/RESUMIR el CONTENIDO de los aportes de los diagnosticos participativos (Consejos de Desarrollo COCODES/COMUDES) en los Planes de Desarrollo Municipal (PDM). Toda la evidencia primaria y secundaria (nota SEGEPLAN ?p=1</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.diariolibre.com/actualidad/nacional/2023/10/11/gobierno-presenta-estrategia-de-inteligencia-artificial/2489157</t>
+          <t>https://portal.segeplan.gob.gt/segeplan/?p=14176</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>LATAM</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Plataforma de modelos generativos de IA de SEGEPLAN + Red Ciudadana (Guatemala)</t>
+          <t>ANTAI Smart CID (Autoridad Nacional de Transparencia y Acceso a la Información + OS City)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Descubrimiento</t>
+          <t>Excluido 2025</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>El criterio ELEGIBLE exige que la IA generativa se use para SISTEMATIZAR/CLASIFICAR/RESUMIR el CONTENIDO de los aportes de los diagnosticos participativos (Consejos de Desarrollo COCODES/COMUDES) en los Planes de Desarrollo Municipal (PDM). Toda la evidencia primaria y secundaria (nota SEGEPLAN ?p=1</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://portal.segeplan.gob.gt/segeplan/?p=14176</t>
+          <t>https://www.caf.com/es/actualidad/noticias/2021/07/caf-realiza-su-primera-inversion-en-una-govtech-latinoamericana/</t>
         </is>
       </c>
     </row>
@@ -6961,7 +7001,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>ANTAI Smart CID (Autoridad Nacional de Transparencia y Acceso a la Información + OS City)</t>
+          <t>Botivist</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -6971,12 +7011,12 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>No tiene foco en un país específico</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.caf.com/es/actualidad/noticias/2021/07/caf-realiza-su-primera-inversion-en-una-govtech-latinoamericana/</t>
+          <t>https://www.microsoft.com/en-us/research/publication/botivist-calling-volunteers-to-action-using-online-bots/</t>
         </is>
       </c>
     </row>
@@ -6988,7 +7028,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Botivist</t>
+          <t>Chatbot DCI (Denuncia Ciudadana Idónea)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -6998,12 +7038,12 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>No tiene foco en un país específico</t>
+          <t>No evidencia de uso de IA</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://www.microsoft.com/en-us/research/publication/botivist-calling-volunteers-to-action-using-online-bots/</t>
+          <t>https://www.policylab.tech/post/revolucionando-la-denuncia-ciudadana-en-am%C3%A9rica-latina-con-tecnolog%C3%ADa-el-caso-del-chatbot-dci-1</t>
         </is>
       </c>
     </row>
@@ -7015,7 +7055,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Chatbot DCI (Denuncia Ciudadana Idónea)</t>
+          <t>Citibeats: Covid-19 (“Percepciones ciudadanas COVID-19”)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -7025,12 +7065,12 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>No evidencia de uso de IA</t>
+          <t>Análisis de redes sociales, no es participación</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://www.policylab.tech/post/revolucionando-la-denuncia-ciudadana-en-am%C3%A9rica-latina-con-tecnolog%C3%ADa-el-caso-del-chatbot-dci-1</t>
+          <t>https://forbescentroamerica.com/2021/04/28/civiclytics-el-big-data-apoya-la-recuperacion-economica</t>
         </is>
       </c>
     </row>
@@ -7042,7 +7082,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Citibeats: Covid-19 (“Percepciones ciudadanas COVID-19”)</t>
+          <t>Ushahidi "AI for Good"</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -7052,24 +7092,24 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Análisis de redes sociales, no es participación</t>
+          <t>No se evidencia el uso de IA en los proyectos de participación listados para Latam</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://forbescentroamerica.com/2021/04/28/civiclytics-el-big-data-apoya-la-recuperacion-economica</t>
+          <t>https://www.ushahidi.com/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>LATAM</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Ushahidi "AI for Good"</t>
+          <t>AMIMgo</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -7079,12 +7119,12 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>No se evidencia el uso de IA en los proyectos de participación listados para Latam</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://www.ushahidi.com/</t>
+          <t>https://amim.mx/noticias/detalle/estrena-amim-chatbot-para-la-atencion-ciudadana</t>
         </is>
       </c>
     </row>
@@ -7096,7 +7136,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>AMIMgo</t>
+          <t>ATIC</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -7106,12 +7146,12 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>https://amim.mx/noticias/detalle/estrena-amim-chatbot-para-la-atencion-ciudadana</t>
+          <t>https://oem.com.mx/la-prensa/metropoli/info-cdmx-implementa-atic-una-herramienta-con-ia-que-facilita-el-acceso-a-la-informacion-13081722</t>
         </is>
       </c>
     </row>
@@ -7123,7 +7163,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>ATIC</t>
+          <t>ChatBot “Claudia"</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -7133,12 +7173,12 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>No es participación</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://oem.com.mx/la-prensa/metropoli/info-cdmx-implementa-atic-una-herramienta-con-ia-que-facilita-el-acceso-a-la-informacion-13081722</t>
+          <t>https://mexicocomovamos.mx/animal-politico/2024/08/chatbot-claudia-una-herramienta-de-participacion-ciudadana/</t>
         </is>
       </c>
     </row>
@@ -7150,7 +7190,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>ChatBot “Claudia"</t>
+          <t>Chatbot "Inés"</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -7160,12 +7200,12 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>No es participación</t>
+          <t>No es participación, es informativo</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>https://mexicocomovamos.mx/animal-politico/2024/08/chatbot-claudia-una-herramienta-de-participacion-ciudadana/</t>
+          <t>https://centralelectoral.ine.mx/2024/04/17/nueva-version-del-chatbot-del-ine-en-whatsapp-permitira-verificar-informacion-sobre-elecciones-2024/</t>
         </is>
       </c>
     </row>
@@ -7177,7 +7217,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Chatbot "Inés"</t>
+          <t>Chatbot Sam Petrino</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -7187,12 +7227,12 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>No es participación, es informativo</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>https://centralelectoral.ine.mx/2024/04/17/nueva-version-del-chatbot-del-ine-en-whatsapp-permitira-verificar-informacion-sobre-elecciones-2024/</t>
+          <t>https://www.civica.digital/historias/chatbot-sam-petrino</t>
         </is>
       </c>
     </row>
@@ -7204,7 +7244,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Chatbot Sam Petrino</t>
+          <t>Chatbot Victoria</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -7219,7 +7259,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>https://www.civica.digital/historias/chatbot-sam-petrino</t>
+          <t>https://adip.cdmx.gob.mx/comunicacion/nota/la-adip-y-el-gobierno-de-la-ciudad-presentan-victoria-el-robot-que-colaborara-en-la-atencion-de-la-ciudadania</t>
         </is>
       </c>
     </row>
@@ -7231,7 +7271,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Chatbot Victoria</t>
+          <t>INAOE (Conacyt) – Laboratorio de Tecnologías del Lenguaje</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -7241,12 +7281,12 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>https://adip.cdmx.gob.mx/comunicacion/nota/la-adip-y-el-gobierno-de-la-ciudad-presentan-victoria-el-robot-que-colaborara-en-la-atencion-de-la-ciudadania</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
     </row>
@@ -7258,22 +7298,22 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>INAOE (Conacyt) – Laboratorio de Tecnologías del Lenguaje</t>
+          <t>Jalisco - Consulta ¡Armemos un Plan! (Plan Estatal de Desarrollo y Gobernanza 2024-2030)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Excluido 2025</t>
+          <t>Excluido (criterio corregido)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>Proceso participativo real y masivo (675.484 participaciones; 15.899 propuestas), pero NO hay evidencia de uso de IA para analizar/agrupar/clasificar el contenido de las propuestas (usa_IA_en_proceso 'no'). Sin uso de IA → NO. Decisión del equipo.</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
+          <t>https://armemosunplan.mx/propuestas-ciudadanas/</t>
         </is>
       </c>
     </row>
@@ -7285,22 +7325,22 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Jalisco - Consulta ¡Armemos un Plan! (Plan Estatal de Desarrollo y Gobernanza 2024-2030)</t>
+          <t>Movimex</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Excluido (criterio corregido)</t>
+          <t>Excluido 2025</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Proceso participativo real y masivo (675.484 participaciones; 15.899 propuestas), pero NO hay evidencia de uso de IA para analizar/agrupar/clasificar el contenido de las propuestas (usa_IA_en_proceso 'no'). Sin uso de IA → NO. Decisión del equipo.</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>https://armemosunplan.mx/propuestas-ciudadanas/</t>
+          <t>https://animalpolitico.com/estados/chatbot-movimex-tramites-denuncias-edomex</t>
         </is>
       </c>
     </row>
@@ -7312,7 +7352,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Movimex</t>
+          <t>Sistema *0311 Locatel</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -7322,12 +7362,12 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>Atención ciudadana</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>https://animalpolitico.com/estados/chatbot-movimex-tramites-denuncias-edomex</t>
+          <t>https://research.latinxinai.org/papers/naacl/2022/pdf/paper_01.pdf</t>
         </is>
       </c>
     </row>
@@ -7339,22 +7379,22 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Sistema *0311 Locatel</t>
+          <t>Sufragio seguro</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Excluido 2025</t>
+          <t>Baseline 2025</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Atención ciudadana</t>
+          <t>EXCLUSIÓN FIRME (recodificación 2026): Exclusión FIRME (recodificación 2026): integridad/proceso electoral, no contenido</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>https://research.latinxinai.org/papers/naacl/2022/pdf/paper_01.pdf</t>
+          <t>https://algoritmoscide.org/proyectos/sufragio-seguro/</t>
         </is>
       </c>
     </row>
@@ -7366,34 +7406,34 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Sufragio seguro</t>
+          <t>Violetta</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Baseline 2025</t>
+          <t>Excluido 2025</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>EXCLUSIÓN FIRME (recodificación 2026): Exclusión FIRME (recodificación 2026): integridad/proceso electoral, no contenido</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>https://algoritmoscide.org/proyectos/sufragio-seguro/</t>
+          <t>https://holasoyvioletta.com/acerca-de/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Violetta</t>
+          <t>Dr. ROSA y Dr. NICO</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -7403,24 +7443,24 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>https://holasoyvioletta.com/acerca-de/</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Dr. ROSA y Dr. NICO</t>
+          <t>JNE WhatsApp Chatbot</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -7435,7 +7475,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
+          <t>https://portal.jne.gob.pe/Portal/Pagina/Nota/12783</t>
         </is>
       </c>
     </row>
@@ -7447,49 +7487,49 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>JNE WhatsApp Chatbot</t>
+          <t>Sistema de cómputo con IA para las Elecciones Generales 2026</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Excluido 2025</t>
+          <t>Excluido (criterio corregido)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>Conteo electoral (OCR de actas): votación política, no participación.</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://portal.jne.gob.pe/Portal/Pagina/Nota/12783</t>
+          <t>https://andina.pe/agencia/noticia-onpe-utilizara-un-nuevo-sistema-computo-resultados-incorporara-ia-1021072.aspx</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PY</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Sistema de cómputo con IA para las Elecciones Generales 2026</t>
+          <t>Consultas ciudadanas sobre IA en Paraguay - PNUD Accelerator Lab (AccLab) + Columbia SIPA + MITIC / insumo del diagnóstico AILA (Atlas de IA)</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Excluido (criterio corregido)</t>
+          <t>Descubrimiento</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Conteo electoral (OCR de actas): votación política, no participación.</t>
+          <t>El criterio ELEGIBLE exige que dentro de un proceso participativo convocado se use IA (NLP/ML/clustering/sentimiento) SOBRE EL CONTENIDO de los aportes. Aquí ocurre lo contrario: (1) la IA es el TEMA de la consulta (se pregunta a la ciudadania por su percepcion de la IA), y (2) el ANÁLISIS de los ap</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://andina.pe/agencia/noticia-onpe-utilizara-un-nuevo-sistema-computo-resultados-incorporara-ia-1021072.aspx</t>
+          <t>https://www.undp.org/es/paraguay/blog/consultas-ciudadanas-sobre-ia-en-paraguay-visiones-diversas-entre-el-campo-y-la-ciudad</t>
         </is>
       </c>
     </row>
@@ -7501,34 +7541,34 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Consultas ciudadanas sobre IA en Paraguay - PNUD Accelerator Lab (AccLab) + Columbia SIPA + MITIC / insumo del diagnóstico AILA (Atlas de IA)</t>
+          <t>ParaEmpleo</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Descubrimiento</t>
+          <t>Excluido 2025</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>El criterio ELEGIBLE exige que dentro de un proceso participativo convocado se use IA (NLP/ML/clustering/sentimiento) SOBRE EL CONTENIDO de los aportes. Aquí ocurre lo contrario: (1) la IA es el TEMA de la consulta (se pregunta a la ciudadania por su percepcion de la IA), y (2) el ANÁLISIS de los ap</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.undp.org/es/paraguay/blog/consultas-ciudadanas-sobre-ia-en-paraguay-visiones-diversas-entre-el-campo-y-la-ciudad</t>
+          <t>https://fairlac.iadb.org/en/paraempleo</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>PY</t>
+          <t>UY</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>ParaEmpleo</t>
+          <t>Chatbot (Asistente virtual entrenado con IA)</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -7538,12 +7578,12 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>https://fairlac.iadb.org/en/paraempleo</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
     </row>
@@ -7555,7 +7595,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Chatbot (Asistente virtual entrenado con IA)</t>
+          <t>Consulta Pública de la Estrategia Nacional de Inteligencia Artificial (IA) de Uruguay 2024–2030,</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -7565,12 +7605,12 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>No evidencia de uso de IA</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
+          <t>https://www.gub.uy/agencia-gobierno-electronico-sociedad-informacion-conocimiento/comunicacion/publicaciones/estrategia-nacional-inteligencia-artificial-2024-2030</t>
         </is>
       </c>
     </row>
@@ -7582,81 +7622,54 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Consulta Pública de la Estrategia Nacional de Inteligencia Artificial (IA) de Uruguay 2024–2030,</t>
+          <t>Consulta Pública y Participación Multiactores: "Niñas, niños, adolescentes, entornos digitales e inteligencia artificial" (Uruguay, 2026)</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Excluido 2025</t>
+          <t>Descubrimiento</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>No evidencia de uso de IA</t>
+          <t>NO (lean firme). (1) TEMPORAL: la consulta está ABIERTA hasta el 10/09/2026 y la fase de sistematización/análisis/validación (Fase 3) recién ocurre entre el 10/09 y el 10/10/2026, con informe final el 30/11/2026. A la fecha de evaluación (2026-07-01) la fase de análisis NO se ha ejecutado, por lo qu</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>https://www.gub.uy/agencia-gobierno-electronico-sociedad-informacion-conocimiento/comunicacion/publicaciones/estrategia-nacional-inteligencia-artificial-2024-2030</t>
+          <t>https://www.gub.uy/ministerio-educacion-cultura/comunicacion/noticias/lanzamiento-consulta-publica-sobre-inteligencia-artificial-entornos-digitales</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>UY</t>
+          <t>VE</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Consulta Pública y Participación Multiactores: "Niñas, niños, adolescentes, entornos digitales e inteligencia artificial" (Uruguay, 2026)</t>
+          <t>Plan de la Patria 7 Transformaciones (7T) - IA y Big Data en la sistematización de propuestas de la Consulta Popular</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Descubrimiento</t>
+          <t>Dudoso</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>NO (lean firme). (1) TEMPORAL: la consulta está ABIERTA hasta el 10/09/2026 y la fase de sistematización/análisis/validación (Fase 3) recién ocurre entre el 10/09 y el 10/10/2026, con informe final el 30/11/2026. A la fecha de evaluación (2026-07-01) la fase de análisis NO se ha ejecutado, por lo qu</t>
+          <t>NO (resuelto en 2ª pasada, antes DUDA). Hay un proceso participativo claro (consulta/debate nacional para construir el Plan de la Patria 7T, con +63.000 asambleas, 3,4 M de participantes y 34.491 propuestas) cuyo CONTENIDO sí fue recolectado, cargado, sistematizado y agrupado. Pero la 2ª pasada CONF</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.gub.uy/ministerio-educacion-cultura/comunicacion/noticias/lanzamiento-consulta-publica-sobre-inteligencia-artificial-entornos-digitales</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>Plan de la Patria 7 Transformaciones (7T) - IA y Big Data en la sistematización de propuestas de la Consulta Popular</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Dudoso</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>NO (resuelto en 2ª pasada, antes DUDA). Hay un proceso participativo claro (consulta/debate nacional para construir el Plan de la Patria 7T, con +63.000 asambleas, 3,4 M de participantes y 34.491 propuestas) cuyo CONTENIDO sí fue recolectado, cargado, sistematizado y agrupado. Pero la 2ª pasada CONF</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
           <t>http://www.correodelorinoco.gob.ve/venezuela-impulsa-el-debate-sobre-inteligencia-artificial-bajo-principios-de-soberania-y-etica/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E74"/>
+  <autoFilter ref="A1:E73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7667,7 +7680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9336,62 +9349,130 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Popular Código de las Familias (GEMA-CEN / XISCOP)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Para agilizar la recogida y el procesamiento de los criterios, la Universidad de las Ciencias Informáticas (UCI) y Datys diseñaron dos sistemas informáticos de gestión (XISCOP y GEMA-CEN) [proceso de consulta popular del Código de las Familias en Cuba].</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>consulta popular del proyecto del Código de las Familias (...) la Universidad de las Ciencias Informáticas (UCI) y Datys diseñaron dos sistemas informáticos de gestión (XISCOP y GEMA-CEN)</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>luego se sube a GEMA-CEN (también operado por especialistas) que, a través del análisis inteligente de los expedientes, organiza las propuestas y agrupa las similares, facilitando el trabajo y evitando errores. GEMA-CEN permite determinar las propuestas típicas para un párrafo en cada una de las categorías establecidas</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Más de seis millones 481 mil personas participaron en las reuniones (...) la consulta popular del proyecto del Código de las Familias (...) convocada entre febrero y abril [de 2022]; del total de propuestas procesadas se determinaron 5 237 propuestas típicas por Título</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>del total de propuestas procesadas se determinaron 5 237 propuestas típicas por Título, conformadas a partir de la asociación de propuestas idénticas y de aquellas con redacción diferente pero referidas al mismo criterio u opinión</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>La consulta popular (...) fue organizada y supervisada por el Consejo Electoral Nacional (CEN) [órgano del Estado cubano]; los resultados se entregaron al Parlamento (Asamblea Nacional) y a su Comisión redactora</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>se sube a GEMA-CEN (...) que, a través del análisis inteligente de los expedientes, organiza las propuestas y agrupa las similares (...) permite determinar las propuestas típicas para un párrafo en cada una de las categorías establecidas</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>GEMA es una herramienta para el análisis de información contenida en grandes volúmenes de archivos de diferentes formatos e idiomas, con funcionalidades orientadas a la recuperación y clasificación de información (...) complementando los resultados mediante técnicas modernas de recuperación de información para obtener archivos similares, eliminar resultados no relevantes y agrupar documentos comunes</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>http://www.datys.cu/spa/site/product/15
+https://www.granma.cu/cuba/2022-01-24/herramientas-digitales-seran-claves-durante-la-consulta-popular-del-codigo-de-las-familias-24-01-2022-13-01-18
+https://www.espirituano.gob.cu/noticias/7716-como-sera-el-proceso-de-consulta-popular-del-nuevo-codigo-de-las-familias
+http://www.cubadebate.cu/noticias/2021/12/19/como-sera-el-proceso-de-consulta-popular-del-nuevo-codigo-de-las-familias/
+http://www.cubadebate.cu/noticias/2022/05/14/consulta-popular-del-proyecto-de-codigo-de-las-familias-61-96-por-ciento-de-opiniones-estuvieron-a-favor/
+https://es.wikipedia.org/wiki/C%C3%B3digo_de_las_Familias_de_Cuba
+https://oncubanews.com/cuba/softwares-cubanos-seran-utilizados-en-el-proceso-de-consulta-popular-sobre-el-codigo-de-las-familias/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>EC</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">PAGA IA </t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Caso del índice ILIA 2025 (BBDD oficial del equipo)</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Referendos e Iniciativas Populares</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Implementación</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>reconfirmado web (institucional): Reconfirmado: integrada al Tercer Plan de Acción de Estado Abierto 2025-2027; analiza las propuestas ciudadanas y sugiere actividades.</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Continuidad (BBDD 2025): Plataforma</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>Gobierno Abierto Ecuador, en colaboración con la Fundación de Ayuda por Internet (Fundapi)</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Analizar temas propuestos y generar sugerencias de compromisos basados en experiencias previas de planes de acción de gobierno abierto
 </t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Analizar temas propuestos y generar sugerencias de compromisos basados en experiencias previas de planes de acción de gobierno abierto
 </t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>https://ia.gobiernoabierto.ec/
 https://ia.gobiernoabierto.ec/
@@ -9399,63 +9480,63 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>GT</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Guatemala Joven Conversa </t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Caso del índice ILIA 2025 (BBDD oficial del equipo)</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>Governanza Colaborativa</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Implementación</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>reconfirmado web (institucional): Reconfirmado: diálogos digitales con IA (DPPA ONU + Fundación Esquipulas); 300+ jóvenes; la IA permite intercambios anónimos y votación de aportes para identifi</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Continuidad (BBDD 2025): Uso único</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>Oficina del Coordinador Residente de las Naciones Unidas en Guatemala y Fundación Esquipulas para la Paz, la Democracia, el Desarrollo y la Integración</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>Facilitar diálogos anónimos en tiempo real, permitir votaciones sobre opiniones y generar alertas sobre desviaciones en la ejecución de obras</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>Facilitar diálogos anónimos en tiempo real, permitir votaciones sobre opiniones y generar alertas sobre desviaciones en la ejecución de obras</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>https://dppa.medium.com/usando-el-poder-de-la-ia-para-impulsar-la-participaci%C3%B3n-pol%C3%ADtica-de-los-j%C3%B3venes-en-guatemala-6f6d7bf45a47
 https://www.fundaesq.org/guatemala-joven-la-voz-de-una-generacion-de-cambios/
@@ -9463,125 +9544,125 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>HN</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RedPública + iVerify </t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Caso del índice ILIA 2025 (BBDD oficial del equipo)</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Referendos e Iniciativas Populares</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Análisis</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>reconfirmado web (institucional): Reverificación: plataforma de propuestas ciudadanas con módulo de análisis de tendencias; evidencia de IA central débil, revisar en Fase 2.</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Continuidad (BBDD 2025): Uso único</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>Programa de las Naciones Unidas para el Desarrollo (PNUD) en colaboración con CEUTEC y la Unión Europea.</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	Detectar y clasificar desinformación electoral antes de su publicación; analizar y agrupar temas de propuestas ciudadanas.</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	Detectar y clasificar desinformación electoral antes de su publicación; analizar y agrupar temas de propuestas ciudadanas.</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.undp.org/es/honduras/historias/participacion-ciudadana-con-innovacion-digital-traves-de-redpublica-honduras</t>
-        </is>
-      </c>
-    </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>HN</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RedPública + iVerify </t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Caso del índice ILIA 2025 (BBDD oficial del equipo)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Referendos e Iniciativas Populares</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Análisis</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>reconfirmado web (institucional): Reverificación: plataforma de propuestas ciudadanas con módulo de análisis de tendencias; evidencia de IA central débil, revisar en Fase 2.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Continuidad (BBDD 2025): Uso único</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Programa de las Naciones Unidas para el Desarrollo (PNUD) en colaboración con CEUTEC y la Unión Europea.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">	Detectar y clasificar desinformación electoral antes de su publicación; analizar y agrupar temas de propuestas ciudadanas.</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">	Detectar y clasificar desinformación electoral antes de su publicación; analizar y agrupar temas de propuestas ciudadanas.</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/es/honduras/historias/participacion-ciudadana-con-innovacion-digital-traves-de-redpublica-honduras</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Guanajuato hará historia con el primer Programa de Gobierno realizado con IA</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Para integrar la participación ciudadana en este Programa de Gobierno, se realizaron cuatro talleres cubriendo las regiones noreste, norte, centro y sur, con representación de los 46 municipios de Guanajuato.</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Recibieron miles de ideas y propuestas, y para asegurar que cada una fuera tomada en cuenta, utilizaron herramientas de inteligencia artificial. Esta tecnología les ayudó a procesar y organizar la información, identificar las prioridades más mencionadas por la ciudadanía y entender las necesidades de cada región. Fue la herramienta que les permitió transformar el gran diálogo social en datos claros para la toma de decisiones.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>El Programa de Gobierno de Guanajuato 2024-2030 es la guía que orienta las acciones del Gobierno de la Gente para lograr un Guanajuato sostenible, equitativo y transparente.</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Su diseño incorporó el uso de inteligencia artificial para integrar más de 26 mil voces de distintas regiones y sectores</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>El Programa de Gobierno 2024-2030 hizo historia al ser el primero en realizarse con ayuda de la Inteligencia Artificial (IA), según anunció la Gobernadora Libia Dennise García Muñoz Ledo en el Consejo de Planeación para el Desarrollo del Estado de Guanajuato (COPLADEG).</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Recibieron miles de ideas y propuestas, y para asegurar que cada una fuera tomada en cuenta, utilizaron herramientas de inteligencia artificial. Esta tecnología les ayudó a procesar y organizar la información, identificar las prioridades más mencionadas por la ciudadanía.</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>Esta tecnología les ayudó a procesar y organizar la información, identificar las prioridades más mencionadas por la ciudadanía y entender las necesidades de cada región. Fue la herramienta que les permitió transformar el gran diálogo social en datos claros para la toma de decisiones.</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>https://guanajuatointeligente.com/como-hicimos-el-programa/
 https://guanajuatointeligente.com/
@@ -9594,121 +9675,121 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Presupuesto CRECES</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Caso del índice ILIA 2025 (BBDD oficial del equipo)</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Presupuestos Participativos</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Implementación</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>BBDD 2025: Activo</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>Continuidad (BBDD 2025): Uso único</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>Ayundamiento de Hermosilla</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Facilitar las votaciones haciéndolo en forma conversacional</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Facilitar las votaciones haciéndolo en forma conversacional</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>https://presupuestocreces.hermosillo.gob.mx/</t>
-        </is>
-      </c>
-    </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Presupuesto CRECES</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Caso del índice ILIA 2025 (BBDD oficial del equipo)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Presupuestos Participativos</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Implementación</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>BBDD 2025: Activo</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Continuidad (BBDD 2025): Uso único</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Ayundamiento de Hermosilla</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Facilitar las votaciones haciéndolo en forma conversacional</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Facilitar las votaciones haciéndolo en forma conversacional</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>https://presupuestocreces.hermosillo.gob.mx/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>La Fundación Panamá Participa lanzó Mansa Idea (www.mansaidea.com), una plataforma basada en inteligencia artificial que recoge miles de propuestas ciudadanas... iniciativa de alcance nacional que se nutre de ideas y propuestas que miles de panameños hicieron durante el desarrollo del Pacto del Bicentenario. (Panamá; fuentes panama24horas.com.pa y laestrella.com.pa)</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Mansa Idea, resultado del Pacto del Bicentenario, ofrece acceso fácil y transparente a más de 175 mil ideas y propuestas generadas por ciudadanos de todo el país. La herramienta digital recoge en un solo clic los consensos nacionales y regionales/provinciales, constituyendo una poderosa base de datos de proyectos con información transparente, 100% confiable y de calidad generada por la ciudadanía.</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Mansa Idea es una plataforma innovadora basada en inteligencia artificial cuyo contenido refleja una inteligencia colectiva que busca construir, a través de miles de propuestas, un mejor futuro para todos. La herramienta digital recoge en un solo clic los consensos nacionales y regionales/provinciales. (la IA agrega/organiza/sintetiza el contenido de las propuestas por tema y territorio = Análisis + Traducción Política; el método técnico exacto no se detalla en las fuentes).</t>
         </is>
       </c>
-      <c r="G32" s="11" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="G33" s="11" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>La plataforma fue lanzada el 1 de abril de 2024... constituye una herramienta valiosa de participación ciudadana muy relevante para ciudadanos, candidatos a cargos de elección popular y medios durante la campaña electoral y luego como recurso para el monitoreo del mandato ciudadano. (un despliegue concreto de la plataforma, 2024; sin evidencia de ediciones recurrentes).</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>La Fundación Panamá Participa lanzó Mansa Idea... iniciativa liderada por Paulina Franceschi a través de la Fundación Panamá Participa (sociedad civil). El proceso participativo de origen: 'El 26 de noviembre de 2020, el presidente Laurentino Cortizo Cohen lanzó la iniciativa denominada Pacto del Bicentenario Cerrando Brechas' (gobierno nacional / Concertación Nacional).</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Mansa Idea es una plataforma innovadora basada en inteligencia artificial cuyo contenido refleja una inteligencia colectiva que busca construir, a través de miles de propuestas, un mejor futuro para todos. (la IA procesa el contenido de las propuestas del proceso participativo).</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>La herramienta digital recoge en un solo clic los consensos nacionales y regionales/provinciales, constituyendo una poderosa base de datos de proyectos con información transparente, 100% confiable y de calidad generada por la ciudadanía. (agregación/síntesis de los aportes ciudadanos = rol sobre el contenido).</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>https://www.panama24horas.com.pa/panama/fundacion-panama-participa-lanza-plataforma-de-propuestas-ciudadanas-mansa-idea/
 https://www.laestrella.com.pa/panama/politica/mansa-idea-una-herramienta-digital-con-propuestas-para-candidatos-YD6746221
@@ -9719,63 +9800,63 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>PE</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Caso del índice ILIA 2025 (BBDD oficial del equipo)</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Governanza Colaborativa</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Análisis</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>reconfirmado web (prensa): VERIFICADO (fuente primaria): el CNE usó IBM Watson Discovery + Studio (ML/NLP) sobre 87.991 documentos de aportes ciudadanos de 847 eventos y 49 espacios de di</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Continuidad (BBDD 2025): Uso único</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>Consejo Nacional de Educación del Perú</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Analizar las opiniones de los participantes y sistematizar la información de forma objetiva.</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Analizar las opiniones de los participantes y sistematizar la información de forma objetiva.</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>https://www.gob.pe/institucion/cne/noticias/502734-lanzan-consulta-ciudadana-por-el-proyecto-educativo-nacional
 https://cdn.www.gob.pe/uploads/document/file/1915017/CNE-%20proyecto-educativo-nacional-al-2036.pdf.pdf?v=1679434080
@@ -9784,59 +9865,59 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>TT</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Project: National Digital Transformation Strategy | Ministry of Digital Transformation, Trinidad and Tobago (engage.gov.tt/projects/national-digital-transformation-strategy). Ruta interna confirmatoria: engage.gov.tt/projects/e-democracy-govocal-internal (la instancia corre sobre Go Vocal). En 2026: 'Projects | Ministry of Public Administration and Artificial Intelligence' (engage.gov.tt/projects).</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>EngageTT es una plataforma en linea (engage.gov.tt) donde ciudadanos, empresas y partes interesadas pueden recibir actualizaciones en tiempo real sobre iniciativas de transformacion digital y ofrecer retroalimentacion via encuestas y sondeos (polls); el Ministro anima a todos a participar y enviar ideas y comentarios sobre el NDTS, que se disena para evolucionar mediante el compromiso y la colaboracion continuos. Incluye un 'Open Forum' (engage.gov.tt/ideas/open-forum) y 'Input: Submitting Proposals' (engage.gov.tt/ideas/submitting-proposals).</t>
         </is>
       </c>
-      <c r="F34" s="11" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>The National Strategy for a Digital TT is finalized, and while the Ministry of Digital Transformation is no longer seeking input, they welcome feedback or comments through the citizen engagement digital platform Engage TT. (engage.gov.tt sigue operativo en 2026 bajo MPAAI).</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>The Ministry of Digital Transformation (MDT) officially presented the National Digital Transformation Strategy (NDTS) 2024-2027... launched during a NDTS Symposium in collaboration with the Inter-American Development Bank (IDB) on Wednesday, February 12th 2025. A major highlight... was the introduction of two new digital tools (EngageTT y AskNDTS). (Lanzamiento/anuncio unico en feb-2025; plataforma de uso continuo pero sin &gt;=2 ediciones de proceso participativo documentadas).</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>The Ministry of Digital Transformation (MDT) officially presented the National Digital Transformation Strategy (NDTS) 2024-2027... and introduced the EngageTT website - an online platform where citizens, businesses, and stakeholders can get real-time updates on digital transformation initiatives, and offer feedback via surveys and polls. (Convocante: gobierno nacional / Ministry of Digital Transformation, hoy MPAAI).</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>Go Vocal Support Base (AI Analysis): 'Access to this feature depends on your plan. Advanced Sensemaking with auto-insights is available in the Premium plan.' -&gt; la IA/NLP de Go Vocal NO es automatica, depende del plan; y para EngageTT solo se documenta 'feedback via surveys and polls'/Open Forum/ideas, SIN mencion de analisis automatico por IA de los aportes. No se halla evidencia de activacion del NLP sobre el contenido en la instancia TT. 3a PASADA (refuerzo): Oxford Insights, 'The country's AI utilisation for citizens is concentrated in a robust Chatbot programme' (mas 'deployment of large language models for internal development purposes') -&gt; la IA ciudadana de TT es el chatbot, NO el analisis de aportes.</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Sin evidencia de IA aplicada al contenido de los aportes en engage.gov.tt. La unica IA confirmada de cara al ciudadano (AskNDTS/ANANSI) es chatbot de FAQ, excluido del criterio. En 3a pasada, el material de MPAAI 2026 enmarca la IA en el asistente ANANSI y en encuestas de AI-readiness (resultados 'consolidated and reviewed' en talleres), sin mencion de analisis por IA de los aportes del NDTS ni de Go Vocal Sensemaking.</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>https://support.govocal.com/en/articles/8316692-ai-analysis
 https://support.govocal.com/en/articles/9015305-faq-on-our-ai-sensemaking-tool
@@ -9858,59 +9939,59 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>UY</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Pol.is en el Referéndum Nacional de la LUC (Uruguay) — equipo UdelaR</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Polis has been used to facilitate discussion and build consensus ... in Uruguay on a national referendum (OCDE 2025, 'Governing with AI')</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>A 13-person team from Uruguay's National University — engineers, communicators, and data scientists — ran Polis alongside the referendum</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>The algorithm maps participants' responses and clusters opinions, facilitating the identification of positions that are supported by the majority of participants (OCDE 2025)</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>16,499 people cast more than 295,000 votes ... The referendum was lost by less than 1%</t>
         </is>
       </c>
-      <c r="H35" s="11" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="H36" s="11" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>A 13-person team from Uruguay's National University — engineers, communicators, and data scientists</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>ran Polis alongside the referendum to look for something deeper than "yes or no"</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Polis revealed that even where public safety divided people, surprising points of consensus broke through on other issues — bridges between groups</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>https://compdemocracy.org/case-studies/2021-uruguay-national-referendum/
 https://www.oecd.org/en/publications/governing-with-artificial-intelligence_795de142-en.html</t>
@@ -9918,7 +9999,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L35"/>
+  <autoFilter ref="A1:L36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9952,7 +10033,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>Planilla con 6 pestañas (criterio corregido). 34 casos entran/dudosos · 73 excluidos · 107 en total. Tras dedup e-Cidadania: 33 iniciativas.</t>
+          <t>Planilla con 6 pestañas (criterio corregido). 35 casos entran/dudosos · 72 excluidos · 107 en total. Tras dedup e-Cidadania: 34 iniciativas.</t>
         </is>
       </c>
     </row>

</xml_diff>